<commit_message>
Add Cyprus plants admin, Esperia/Linyang docs, RTB intelligence, and trading bot.
Includes prospect/plant APIs, CERA enrichment scripts, commercial guides, guarantee drafts, and stochrsi paper-trading scaffold alongside ongoing LOI and portfolio updates.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/internal/Lighthief-EPC-Confirmed-Adders-v5-May2026.xlsx
+++ b/docs/internal/Lighthief-EPC-Confirmed-Adders-v5-May2026.xlsx
@@ -5471,39 +5471,39 @@
     <row r="9">
       <c r="A9" s="32" t="inlineStr">
         <is>
-          <t>LV Cabling (DC side)</t>
+          <t>LV+MV+DC Cabling (Joha Cable)</t>
         </is>
       </c>
       <c r="B9" s="32" t="inlineStr">
         <is>
-          <t>€1,400 / BESS container (avg)</t>
+          <t>Per-park lump sum — see v4 Excel column</t>
         </is>
       </c>
       <c r="C9" s="32" t="inlineStr">
         <is>
-          <t>Internal estimate</t>
+          <t>Joha Cable</t>
         </is>
       </c>
       <c r="D9" s="32" t="inlineStr">
         <is>
-          <t>ESTIMATE</t>
+          <t>QUOTED</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="32" t="inlineStr">
         <is>
-          <t>MV Cabling (external)</t>
+          <t xml:space="preserve">  (fallback model if no park line)</t>
         </is>
       </c>
       <c r="B10" s="32" t="inlineStr">
         <is>
-          <t>€3,500 / MV skid</t>
+          <t>€1,400 / BESS + €3,500 / MV skid</t>
         </is>
       </c>
       <c r="C10" s="32" t="inlineStr">
         <is>
-          <t>Internal estimate</t>
+          <t>Internal — do not use for margin</t>
         </is>
       </c>
       <c r="D10" s="32" t="inlineStr">
@@ -5525,7 +5525,7 @@
       </c>
       <c r="C11" s="32" t="inlineStr">
         <is>
-          <t>Internal estimate</t>
+          <t>TBC — confirm vs Joha quote</t>
         </is>
       </c>
       <c r="D11" s="32" t="inlineStr">

</xml_diff>

<commit_message>
SSOT: Galascope Kouklis concrete bases quote (€98,420), updated margins to 10.95%
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/internal/Lighthief-EPC-Confirmed-Adders-v5-May2026.xlsx
+++ b/docs/internal/Lighthief-EPC-Confirmed-Adders-v5-May2026.xlsx
@@ -915,7 +915,7 @@
         <v>1600</v>
       </c>
       <c r="AB3" s="10" t="n">
-        <v>40000</v>
+        <v>65435</v>
       </c>
       <c r="AC3" s="10" t="n">
         <v>13865.34</v>
@@ -924,7 +924,7 @@
         <v>7000</v>
       </c>
       <c r="AE3" s="6" t="n">
-        <v>154585.46</v>
+        <v>180020.46</v>
       </c>
       <c r="AF3" s="6" t="n">
         <v>22897</v>
@@ -939,16 +939,16 @@
         <v>97897</v>
       </c>
       <c r="AJ3" s="13" t="n">
-        <v>2101194.89</v>
+        <v>2126629.89</v>
       </c>
       <c r="AK3" s="13" t="n">
-        <v>2258900</v>
+        <v>2238000</v>
       </c>
       <c r="AL3" s="13" t="n">
-        <v>157705.1100000003</v>
+        <v>111370.1100000003</v>
       </c>
       <c r="AM3" s="14" t="n">
-        <v>0.0698150028775069</v>
+        <v>0.04976323056300283</v>
       </c>
     </row>
     <row r="4">
@@ -1044,7 +1044,7 @@
         <v>1600</v>
       </c>
       <c r="AB4" s="10" t="n">
-        <v>20000</v>
+        <v>32985</v>
       </c>
       <c r="AC4" s="10" t="n">
         <v>7308.43</v>
@@ -1053,7 +1053,7 @@
         <v>7000</v>
       </c>
       <c r="AE4" s="6" t="n">
-        <v>93515.97999999998</v>
+        <v>106500.98</v>
       </c>
       <c r="AF4" s="6" t="n">
         <v>15141</v>
@@ -1068,16 +1068,16 @@
         <v>30141</v>
       </c>
       <c r="AJ4" s="13" t="n">
-        <v>1098113.98</v>
+        <v>1111098.98</v>
       </c>
       <c r="AK4" s="13" t="n">
         <v>1206300</v>
       </c>
       <c r="AL4" s="13" t="n">
-        <v>108186.02</v>
+        <v>95201.02000000002</v>
       </c>
       <c r="AM4" s="14" t="n">
-        <v>0.08968417474923321</v>
+        <v>0.07891985409931196</v>
       </c>
     </row>
     <row r="5">
@@ -4830,22 +4830,22 @@
         <v>2823169.43</v>
       </c>
       <c r="G2" s="20" t="n">
-        <v>248101.44</v>
+        <v>286521.4399999999</v>
       </c>
       <c r="H2" s="20" t="n">
         <v>128038</v>
       </c>
       <c r="I2" s="20" t="n">
-        <v>3199308.87</v>
+        <v>3237728.87</v>
       </c>
       <c r="J2" s="22" t="n">
-        <v>3465200</v>
+        <v>3444300</v>
       </c>
       <c r="K2" s="22" t="n">
-        <v>265891.1300000004</v>
+        <v>206571.1300000004</v>
       </c>
       <c r="L2" s="23" t="n">
-        <v>0.07673182788872225</v>
+        <v>0.05997477861974868</v>
       </c>
       <c r="M2" s="22" t="n">
         <v>12000</v>
@@ -5285,22 +5285,22 @@
         <v>50793042.88</v>
       </c>
       <c r="G11" s="28" t="n">
-        <v>4316471.239999999</v>
+        <v>4354891.239999999</v>
       </c>
       <c r="H11" s="28" t="n">
         <v>1641264</v>
       </c>
       <c r="I11" s="28" t="n">
-        <v>56750778.12</v>
+        <v>56789198.12</v>
       </c>
       <c r="J11" s="28" t="n">
-        <v>64922622</v>
+        <v>64901722</v>
       </c>
       <c r="K11" s="28" t="n">
-        <v>8171843.88</v>
+        <v>8112523.88</v>
       </c>
       <c r="L11" s="30" t="n">
-        <v>0.1258705152111694</v>
+        <v>0.1249970513879431</v>
       </c>
       <c r="M11" s="28" t="n">
         <v>209400</v>
@@ -5838,17 +5838,17 @@
       </c>
       <c r="B28" s="32" t="inlineStr">
         <is>
-          <t>€2,000 / MWh all-in  (Kamil confirmed Feb 2026)</t>
+          <t>€2,000 / MWh default; Galascope Kouklis €98,420 bases (16 Jun 2026); Galascope trenches client-paid</t>
         </is>
       </c>
       <c r="C28" s="32" t="inlineStr">
         <is>
-          <t>Kamil / subcontractors</t>
+          <t>Kouklis / subcontractors</t>
         </is>
       </c>
       <c r="D28" s="32" t="inlineStr">
         <is>
-          <t>CONFIRMED</t>
+          <t>QUOTED-GALASCOPE</t>
         </is>
       </c>
     </row>

</xml_diff>